<commit_message>
final runs number 7
</commit_message>
<xml_diff>
--- a/Data/management_strategy.xlsx
+++ b/Data/management_strategy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Multispecies_model\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F2D02F-ABC2-4749-AABC-C4D1712E3BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF0AD46-A63E-47BC-8BFE-F8BC12CFDB41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-16110" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{532DA4F2-2DD5-4820-8FAD-AC4589CD9F3F}"/>
+    <workbookView xWindow="-26280" yWindow="-13875" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{532DA4F2-2DD5-4820-8FAD-AC4589CD9F3F}"/>
   </bookViews>
   <sheets>
     <sheet name="How_to" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="81">
   <si>
     <t>Stock</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>troph.cat</t>
+  </si>
+  <si>
+    <t>mean</t>
   </si>
 </sst>
 </file>
@@ -808,13 +811,13 @@
         <v>0</v>
       </c>
       <c r="H2" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I2" s="9">
         <v>1</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>48</v>
@@ -852,13 +855,13 @@
         <v>0</v>
       </c>
       <c r="H3" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I3" s="9">
         <v>1</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>49</v>
@@ -896,13 +899,13 @@
         <v>0</v>
       </c>
       <c r="H4" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I4" s="9">
         <v>1</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>48</v>
@@ -940,13 +943,13 @@
         <v>0</v>
       </c>
       <c r="H5" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I5" s="9">
         <v>1</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>50</v>
@@ -984,13 +987,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I6" s="9">
         <v>1</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>48</v>
@@ -1028,13 +1031,13 @@
         <v>0</v>
       </c>
       <c r="H7" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I7" s="9">
         <v>1</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>51</v>
@@ -1072,13 +1075,13 @@
         <v>0</v>
       </c>
       <c r="H8" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I8" s="9">
         <v>1</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>52</v>
@@ -1116,13 +1119,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I9" s="9">
         <v>1</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>53</v>
@@ -1160,13 +1163,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I10" s="9">
         <v>1</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>54</v>
@@ -1204,13 +1207,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I11" s="9">
         <v>1</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>55</v>
@@ -1248,13 +1251,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I12" s="9">
         <v>1</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>56</v>
@@ -1292,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I13" s="9">
         <v>1</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>57</v>
@@ -1336,13 +1339,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I14" s="9">
         <v>1</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>54</v>
@@ -1380,13 +1383,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I15" s="9">
         <v>1</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>57</v>
@@ -1424,13 +1427,13 @@
         <v>0</v>
       </c>
       <c r="H16" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I16" s="9">
         <v>1</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>58</v>
@@ -1468,13 +1471,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I17" s="9">
         <v>1</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>58</v>
@@ -1512,13 +1515,13 @@
         <v>0</v>
       </c>
       <c r="H18" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I18" s="9">
         <v>1</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>58</v>
@@ -1556,13 +1559,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I19" s="9">
         <v>1</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>59</v>
@@ -1600,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="9">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I20" s="9">
         <v>1</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>60</v>

</xml_diff>